<commit_message>
mise à jour du tab
</commit_message>
<xml_diff>
--- a/assets/pdf/Tableau_portfolio_E5.xlsx
+++ b/assets/pdf/Tableau_portfolio_E5.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t xml:space="preserve">BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -123,6 +123,15 @@
   </si>
   <si>
     <t xml:space="preserve">SpaceHub : entreprise fictive de location de lieux On a développé un site internet en Symfony.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wordpress en première année, on a fait un Gantt pour travailler en groupe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profil LinkedIN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portfolio</t>
   </si>
   <si>
     <t xml:space="preserve">Réalisations en milieu professionnel en cours de première année</t>
@@ -639,16 +648,16 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="3" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1080,42 +1089,48 @@
         <v>26</v>
       </c>
       <c r="B10" s="20"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
       <c r="E10" s="24"/>
       <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
+      <c r="G10" s="24"/>
       <c r="H10" s="23"/>
     </row>
     <row r="11" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19"/>
+      <c r="A11" s="19" t="s">
+        <v>27</v>
+      </c>
       <c r="B11" s="20"/>
       <c r="C11" s="22"/>
       <c r="D11" s="22"/>
       <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
+      <c r="F11" s="24"/>
       <c r="G11" s="22"/>
       <c r="H11" s="23"/>
     </row>
     <row r="12" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19"/>
+      <c r="A12" s="19" t="s">
+        <v>28</v>
+      </c>
       <c r="B12" s="20"/>
       <c r="C12" s="22"/>
       <c r="D12" s="22"/>
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
       <c r="G12" s="22"/>
-      <c r="H12" s="23"/>
+      <c r="H12" s="25"/>
     </row>
     <row r="13" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19"/>
+      <c r="A13" s="19" t="s">
+        <v>29</v>
+      </c>
       <c r="B13" s="20"/>
-      <c r="C13" s="22"/>
+      <c r="C13" s="24"/>
       <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
+      <c r="E13" s="24"/>
       <c r="F13" s="22"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="23"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="25"/>
     </row>
     <row r="14" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="19"/>
@@ -1168,20 +1183,20 @@
       <c r="H18" s="23"/>
     </row>
     <row r="19" s="17" customFormat="true" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="25"/>
+      <c r="A19" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
     </row>
     <row r="20" s="17" customFormat="true" ht="176.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="26" t="s">
-        <v>28</v>
+      <c r="A20" s="27" t="s">
+        <v>31</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="22"/>
@@ -1192,8 +1207,8 @@
       <c r="H20" s="23"/>
     </row>
     <row r="21" s="17" customFormat="true" ht="216.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="26" t="s">
-        <v>29</v>
+      <c r="A21" s="27" t="s">
+        <v>32</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="22"/>
@@ -1201,11 +1216,11 @@
       <c r="E21" s="24"/>
       <c r="F21" s="24"/>
       <c r="G21" s="24"/>
-      <c r="H21" s="27"/>
+      <c r="H21" s="25"/>
     </row>
     <row r="22" s="17" customFormat="true" ht="207.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="26" t="s">
-        <v>30</v>
+      <c r="A22" s="27" t="s">
+        <v>33</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="24"/>
@@ -1216,20 +1231,20 @@
       <c r="H22" s="23"/>
     </row>
     <row r="23" s="17" customFormat="true" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25"/>
-      <c r="H23" s="25"/>
+      <c r="A23" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="B23" s="26"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
     </row>
     <row r="24" s="17" customFormat="true" ht="143.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="26" t="s">
-        <v>32</v>
+      <c r="A24" s="27" t="s">
+        <v>35</v>
       </c>
       <c r="B24" s="20"/>
       <c r="C24" s="24"/>
@@ -1240,8 +1255,8 @@
       <c r="H24" s="23"/>
     </row>
     <row r="25" s="17" customFormat="true" ht="324.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="26" t="s">
-        <v>33</v>
+      <c r="A25" s="27" t="s">
+        <v>36</v>
       </c>
       <c r="B25" s="20"/>
       <c r="C25" s="24"/>
@@ -1249,10 +1264,10 @@
       <c r="E25" s="24"/>
       <c r="F25" s="24"/>
       <c r="G25" s="24"/>
-      <c r="H25" s="27"/>
+      <c r="H25" s="25"/>
     </row>
     <row r="26" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="26"/>
+      <c r="A26" s="27"/>
       <c r="B26" s="20"/>
       <c r="C26" s="22"/>
       <c r="D26" s="22"/>
@@ -1262,7 +1277,7 @@
       <c r="H26" s="23"/>
     </row>
     <row r="27" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="26"/>
+      <c r="A27" s="27"/>
       <c r="B27" s="20"/>
       <c r="C27" s="22"/>
       <c r="D27" s="22"/>

</xml_diff>